<commit_message>
Ajout APIs transactions, disputes, gestion d'erreurs + .gitignore
</commit_message>
<xml_diff>
--- a/docs/Suivi_Projet_PFE_Dispute_Chargeback (1).xlsx
+++ b/docs/Suivi_Projet_PFE_Dispute_Chargeback (1).xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\OneDrive\stage_pfa hps\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\OneDrive\stage_pfa hps\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -1163,10 +1163,10 @@
         <v>14</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>16</v>
+        <v>93</v>
       </c>
       <c r="H14" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="25" x14ac:dyDescent="0.35">
@@ -1189,10 +1189,10 @@
         <v>27</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>16</v>
+        <v>93</v>
       </c>
       <c r="H15" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">

</xml_diff>